<commit_message>
Ajuste de Top 5 y Sedes Mayo
</commit_message>
<xml_diff>
--- a/Tabla de Puntos.xlsx
+++ b/Tabla de Puntos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://smileag-my.sharepoint.com/personal/marco_herrero_smileag_mx/Documents/Documents/Procter/Juntas Mensuales/Mayo 26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marco Herrero\Desktop\Dashboard_Torneo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{52B1E4E2-A42B-4D44-85E5-C256B4284837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CCAD23E-47E4-4AAD-95A6-C8A41B79E4DA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC73ACAD-C47D-4D7C-9F68-B8237FBDA9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="3555" windowWidth="29040" windowHeight="15720" xr2:uid="{C4FCA752-2950-48C0-A124-A1B14B3A1160}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
   <si>
     <t>Numero</t>
   </si>
@@ -213,6 +213,9 @@
   </si>
   <si>
     <t>Total puntos Abril</t>
+  </si>
+  <si>
+    <t>Total puntos Mayo</t>
   </si>
 </sst>
 </file>
@@ -657,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19309B8B-C256-401C-B289-2D6397679E35}">
-  <dimension ref="A2:O40"/>
+  <dimension ref="A2:T40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.36328125" customWidth="1"/>
@@ -666,9 +669,11 @@
     <col min="10" max="10" width="17.453125" customWidth="1"/>
     <col min="12" max="12" width="13.1796875" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
+    <col min="18" max="18" width="14.36328125" customWidth="1"/>
+    <col min="20" max="20" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -714,8 +719,23 @@
       <c r="O2" s="8" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="P2" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -759,7 +779,7 @@
         <v>46.78</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -803,7 +823,7 @@
         <v>44.010000000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -847,7 +867,7 @@
         <v>46.06</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -891,7 +911,7 @@
         <v>47.269999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -935,7 +955,7 @@
         <v>45.56</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -982,7 +1002,7 @@
         <v>68.800000000000011</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -1026,7 +1046,7 @@
         <v>46.46</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>48</v>
       </c>
@@ -1073,7 +1093,7 @@
         <v>50.42</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1120,7 +1140,7 @@
         <v>70.44</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -1167,7 +1187,7 @@
         <v>72.44</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -1211,7 +1231,7 @@
         <v>41.51</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -1255,7 +1275,7 @@
         <v>40.67</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -1300,7 +1320,7 @@
         <v>52.15</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>50</v>
       </c>

</xml_diff>